<commit_message>
Tree updates (5/22/25 draft)
</commit_message>
<xml_diff>
--- a/analyses/trees/Chaq/Chaq_Seq_IDs.xlsx
+++ b/analyses/trees/Chaq/Chaq_Seq_IDs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lexikeene/Documents/Research/diverse_collections/github/analyses/trees/Chaq/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E15F4F23-1FA1-9544-8285-D1F550E9165B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A004BB2B-DCEC-D643-BED5-4435E5D229DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33080" yWindow="500" windowWidth="15880" windowHeight="19400" xr2:uid="{CABCAD94-9EAC-A04D-81FC-60523DFF2B09}"/>
+    <workbookView xWindow="33080" yWindow="500" windowWidth="22520" windowHeight="19400" xr2:uid="{CABCAD94-9EAC-A04D-81FC-60523DFF2B09}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="242">
   <si>
     <t>D_mel_USA_2021_mel-21-MDS-9_Chaq_virus_Complete_CDS</t>
   </si>
@@ -588,6 +588,180 @@
   </si>
   <si>
     <t>PV185880</t>
+  </si>
+  <si>
+    <t>sample_id</t>
+  </si>
+  <si>
+    <t>mel-21-MDS-9</t>
+  </si>
+  <si>
+    <t>500-F-11</t>
+  </si>
+  <si>
+    <t>500-F-41</t>
+  </si>
+  <si>
+    <t>500-M-17</t>
+  </si>
+  <si>
+    <t>500-M-57</t>
+  </si>
+  <si>
+    <t>500-M-61-2</t>
+  </si>
+  <si>
+    <t>500-M-61</t>
+  </si>
+  <si>
+    <t>500-M-65-2</t>
+  </si>
+  <si>
+    <t>500-M-65</t>
+  </si>
+  <si>
+    <t>500-M-71-2</t>
+  </si>
+  <si>
+    <t>500-M-84</t>
+  </si>
+  <si>
+    <t>500-M-F10</t>
+  </si>
+  <si>
+    <t>1020-A7</t>
+  </si>
+  <si>
+    <t>1020-B6</t>
+  </si>
+  <si>
+    <t>1020-D3</t>
+  </si>
+  <si>
+    <t>1020-F6</t>
+  </si>
+  <si>
+    <t>1020-F-31</t>
+  </si>
+  <si>
+    <t>1020-F-40</t>
+  </si>
+  <si>
+    <t>1020-F-0818-D4</t>
+  </si>
+  <si>
+    <t>1020-M-19</t>
+  </si>
+  <si>
+    <t>1020-M-0818-A5</t>
+  </si>
+  <si>
+    <t>1020-M-0818-A7</t>
+  </si>
+  <si>
+    <t>1428-F-8</t>
+  </si>
+  <si>
+    <t>1428-M-4</t>
+  </si>
+  <si>
+    <t>1428-M-42</t>
+  </si>
+  <si>
+    <t>Adobe-B8</t>
+  </si>
+  <si>
+    <t>Briarwood-D9</t>
+  </si>
+  <si>
+    <t>CVID-0911-F4</t>
+  </si>
+  <si>
+    <t>CVID-1006-G6</t>
+  </si>
+  <si>
+    <t>CVID-1006-G7</t>
+  </si>
+  <si>
+    <t>CVID-1006-H2</t>
+  </si>
+  <si>
+    <t>CVID-1006-H3</t>
+  </si>
+  <si>
+    <t>James-A5</t>
+  </si>
+  <si>
+    <t>ME-F-1</t>
+  </si>
+  <si>
+    <t>ME-F-2</t>
+  </si>
+  <si>
+    <t>ME-F-3</t>
+  </si>
+  <si>
+    <t>ME-M-1</t>
+  </si>
+  <si>
+    <t>ME-M-2</t>
+  </si>
+  <si>
+    <t>ME-M-7</t>
+  </si>
+  <si>
+    <t>ME-M-8</t>
+  </si>
+  <si>
+    <t>ME-M-11</t>
+  </si>
+  <si>
+    <t>Myrtle-E9</t>
+  </si>
+  <si>
+    <t>OH-M-5</t>
+  </si>
+  <si>
+    <t>Peach-13-H7</t>
+  </si>
+  <si>
+    <t>Penn-F-1</t>
+  </si>
+  <si>
+    <t>Penn-F-2</t>
+  </si>
+  <si>
+    <t>Penn-F-3</t>
+  </si>
+  <si>
+    <t>Penn-F-4</t>
+  </si>
+  <si>
+    <t>Penn-F-6</t>
+  </si>
+  <si>
+    <t>Penn-F-9</t>
+  </si>
+  <si>
+    <t>Penn-F-12</t>
+  </si>
+  <si>
+    <t>Penn-M-2</t>
+  </si>
+  <si>
+    <t>Penn-M-8</t>
+  </si>
+  <si>
+    <t>Penn-M-10</t>
+  </si>
+  <si>
+    <t>Penn-M-11</t>
+  </si>
+  <si>
+    <t>Penn-M-14</t>
+  </si>
+  <si>
+    <t>ME-M-3</t>
   </si>
 </sst>
 </file>
@@ -959,14 +1133,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98BE16B9-83EF-2E42-A6CA-A756C8FEFDB1}">
-  <dimension ref="A1:E107"/>
+  <dimension ref="A1:F107"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="54" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>167</v>
       </c>
@@ -982,8 +1157,11 @@
       <c r="E1" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -999,8 +1177,11 @@
       <c r="E2" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F2" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1016,8 +1197,11 @@
       <c r="E3" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F3" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1033,8 +1217,11 @@
       <c r="E4" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F4" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -1050,8 +1237,11 @@
       <c r="E5" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F5" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1067,8 +1257,11 @@
       <c r="E6" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F6" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -1084,8 +1277,11 @@
       <c r="E7" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F7" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -1101,8 +1297,11 @@
       <c r="E8" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F8" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -1118,8 +1317,11 @@
       <c r="E9" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F9" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1135,8 +1337,11 @@
       <c r="E10" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F10" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -1152,8 +1357,11 @@
       <c r="E11" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F11" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -1169,8 +1377,11 @@
       <c r="E12" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F12" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1186,8 +1397,11 @@
       <c r="E13" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F13" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -1203,8 +1417,11 @@
       <c r="E14" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F14" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -1220,8 +1437,11 @@
       <c r="E15" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F15" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -1237,8 +1457,11 @@
       <c r="E16" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F16" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -1254,8 +1477,11 @@
       <c r="E17" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F17" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -1271,8 +1497,11 @@
       <c r="E18" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F18" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>34</v>
       </c>
@@ -1288,8 +1517,11 @@
       <c r="E19" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F19" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>36</v>
       </c>
@@ -1305,8 +1537,11 @@
       <c r="E20" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F20" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>38</v>
       </c>
@@ -1322,8 +1557,11 @@
       <c r="E21" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F21" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -1339,8 +1577,11 @@
       <c r="E22" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F22" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>42</v>
       </c>
@@ -1356,8 +1597,11 @@
       <c r="E23" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F23" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>44</v>
       </c>
@@ -1373,8 +1617,11 @@
       <c r="E24" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F24" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>46</v>
       </c>
@@ -1390,8 +1637,11 @@
       <c r="E25" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F25" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>48</v>
       </c>
@@ -1407,8 +1657,11 @@
       <c r="E26" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F26" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>50</v>
       </c>
@@ -1424,8 +1677,11 @@
       <c r="E27" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F27" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>52</v>
       </c>
@@ -1441,8 +1697,11 @@
       <c r="E28" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F28" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>54</v>
       </c>
@@ -1458,8 +1717,11 @@
       <c r="E29" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F29" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>56</v>
       </c>
@@ -1475,8 +1737,11 @@
       <c r="E30" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F30" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>58</v>
       </c>
@@ -1492,8 +1757,11 @@
       <c r="E31" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F31" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>60</v>
       </c>
@@ -1509,8 +1777,11 @@
       <c r="E32" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F32" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>62</v>
       </c>
@@ -1526,8 +1797,11 @@
       <c r="E33" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F33" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>64</v>
       </c>
@@ -1543,8 +1817,11 @@
       <c r="E34" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F34" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>66</v>
       </c>
@@ -1560,8 +1837,11 @@
       <c r="E35" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F35" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>68</v>
       </c>
@@ -1577,8 +1857,11 @@
       <c r="E36" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F36" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>70</v>
       </c>
@@ -1594,8 +1877,11 @@
       <c r="E37" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F37" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>72</v>
       </c>
@@ -1611,8 +1897,11 @@
       <c r="E38" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F38" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>74</v>
       </c>
@@ -1628,8 +1917,11 @@
       <c r="E39" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F39" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>76</v>
       </c>
@@ -1645,8 +1937,11 @@
       <c r="E40" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F40" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>78</v>
       </c>
@@ -1662,8 +1957,11 @@
       <c r="E41" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F41" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>80</v>
       </c>
@@ -1679,8 +1977,11 @@
       <c r="E42" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F42" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>82</v>
       </c>
@@ -1696,8 +1997,11 @@
       <c r="E43" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F43" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>84</v>
       </c>
@@ -1713,8 +2017,11 @@
       <c r="E44" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F44" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>86</v>
       </c>
@@ -1730,8 +2037,11 @@
       <c r="E45" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F45" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>88</v>
       </c>
@@ -1747,8 +2057,11 @@
       <c r="E46" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F46" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>90</v>
       </c>
@@ -1764,8 +2077,11 @@
       <c r="E47" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F47" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>92</v>
       </c>
@@ -1781,8 +2097,11 @@
       <c r="E48" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F48" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>94</v>
       </c>
@@ -1798,8 +2117,11 @@
       <c r="E49" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F49" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>96</v>
       </c>
@@ -1815,8 +2137,11 @@
       <c r="E50" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F50" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>98</v>
       </c>
@@ -1832,8 +2157,11 @@
       <c r="E51" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F51" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>100</v>
       </c>
@@ -1849,8 +2177,11 @@
       <c r="E52" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F52" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>102</v>
       </c>
@@ -1866,8 +2197,11 @@
       <c r="E53" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F53" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>104</v>
       </c>
@@ -1883,8 +2217,11 @@
       <c r="E54" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F54" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>106</v>
       </c>
@@ -1900,8 +2237,11 @@
       <c r="E55" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F55" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>108</v>
       </c>
@@ -1917,8 +2257,11 @@
       <c r="E56" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F56" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>110</v>
       </c>
@@ -1934,8 +2277,11 @@
       <c r="E57" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F57" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>112</v>
       </c>
@@ -1951,8 +2297,11 @@
       <c r="E58" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F58" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>114</v>
       </c>
@@ -1968,8 +2317,11 @@
       <c r="E59" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F59" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>116</v>
       </c>
@@ -1985,8 +2337,11 @@
       <c r="E60" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F60" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>118</v>
       </c>
@@ -2002,8 +2357,11 @@
       <c r="E61" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F61" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>120</v>
       </c>
@@ -2019,8 +2377,11 @@
       <c r="E62" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F62" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B63" t="s">
         <v>122</v>
       </c>
@@ -2034,7 +2395,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B64" t="s">
         <v>123</v>
       </c>

</xml_diff>